<commit_message>
Update other iteration 1 docs
</commit_message>
<xml_diff>
--- a/doc/CS673_SPPP_RiskManagement_team1.xlsx
+++ b/doc/CS673_SPPP_RiskManagement_team1.xlsx
@@ -13,10 +13,16 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={3537aad7-61ec-4174-8bf4-ac3232dc566f}</author>
+    <author/>
+    <author>tc={3450403c-4910-4d2c-94df-cc317855ebaa}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{3537aad7-61ec-4174-8bf4-ac3232dc566f}" ref="F13">
+    <comment authorId="0" ref="A10">
+      <text>
+        <t xml:space="preserve">New risk register for iteration 1</t>
+      </text>
+    </comment>
+    <comment authorId="1" xr:uid="{3450403c-4910-4d2c-94df-cc317855ebaa}" ref="F14">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -30,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="107">
   <si>
     <t>This sheet provides some common risks in student projects. You should check if it applies to your group project. 
 You should also feel free to add other risks. Exemplary analysis is also added.</t>
@@ -79,7 +85,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t xml:space="preserve">personel </t>
+    <t>Personel</t>
   </si>
   <si>
     <t>Loss team members</t>
@@ -175,6 +181,15 @@
     <t>Add linter into source code, agree on coding conventions, and review changes through pull requests.</t>
   </si>
   <si>
+    <t>multiple toolings</t>
+  </si>
+  <si>
+    <t>Share documentations in multiple platforms including Discord, Drive, and Git leading to hard to keep track of and someone might get access to</t>
+  </si>
+  <si>
+    <t>Consolidate tools by using Discord for chat only, drive for live documentations, and Github for source code and final documentation or read me file.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Requirements </t>
   </si>
   <si>
@@ -350,12 +365,6 @@
   </si>
   <si>
     <t>Setup CI/CD as soon as the project getting started</t>
-  </si>
-  <si>
-    <t>The team member who is adding the new feature should be the one who determines what is correct for the new functionality that was added.</t>
-  </si>
-  <si>
-    <t>Work together as a team to make sure each developer has the same environment. This is useful so that there aren't accidental bugs added due to environment issues.</t>
   </si>
 </sst>
 </file>
@@ -366,7 +375,7 @@
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="165" formatCode="m/d"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -383,8 +392,11 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <color rgb="FF000000"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -397,17 +409,20 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAD3"/>
+        <bgColor rgb="FFD9EAD3"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border/>
-    <border>
-      <right/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="26">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -441,6 +456,27 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="right" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -462,11 +498,8 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -486,13 +519,13 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Kimleng Lim" id="{60b317be-9454-4f1a-80f1-565478cfa294}" providerId="google-sheets"/>
+  <x18tc:person displayName="Kimleng Lim" id="{a47ff001-7b71-463f-814a-e894643890ca}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="F13" dT="2026-09-07T19:06:17.00" personId="{60b317be-9454-4f1a-80f1-565478cfa294}" id="{3537aad7-61ec-4174-8bf4-ac3232dc566f}" done="0">
+  <x18tc:threadedComment ref="F14" dT="2026-09-07T19:06:17.00" personId="{a47ff001-7b71-463f-814a-e894643890ca}" id="{3450403c-4910-4d2c-94df-cc317855ebaa}" done="0">
     <x18tc:text xml:space="preserve">It's costly because it can lead to team member dropping out.</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -591,7 +624,7 @@
         <v>4.0</v>
       </c>
       <c r="G3" s="4">
-        <f t="shared" ref="G3:G25" si="1">(6-D3)*(6-E3)*F3</f>
+        <f t="shared" ref="G3:G26" si="1">(6-D3)*(6-E3)*F3</f>
         <v>20</v>
       </c>
       <c r="H3" s="3" t="s">
@@ -928,80 +961,80 @@
       <c r="AA9" s="6"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="11"/>
+      <c r="B10" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="E10" s="13">
+        <v>3.0</v>
+      </c>
+      <c r="F10" s="13">
+        <v>2.0</v>
+      </c>
+      <c r="G10" s="14">
+        <f t="shared" si="1"/>
+        <v>24</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I10" s="15">
+        <v>46304.0</v>
+      </c>
+      <c r="J10" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="4">
+      <c r="K10" s="16"/>
+      <c r="L10" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="M10" s="17"/>
+      <c r="N10" s="17"/>
+      <c r="O10" s="17"/>
+      <c r="P10" s="17"/>
+      <c r="Q10" s="17"/>
+      <c r="R10" s="17"/>
+      <c r="S10" s="17"/>
+      <c r="T10" s="17"/>
+      <c r="U10" s="17"/>
+      <c r="V10" s="17"/>
+      <c r="W10" s="17"/>
+      <c r="X10" s="17"/>
+      <c r="Y10" s="17"/>
+      <c r="Z10" s="17"/>
+      <c r="AA10" s="17"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="4">
         <v>1.0</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E11" s="4">
         <v>5.0</v>
       </c>
-      <c r="F10" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="G10" s="8">
+      <c r="F11" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="G11" s="8">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="H10" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I10" s="5">
-        <v>46304.0</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="K10" s="7"/>
-      <c r="L10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="6"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="6"/>
-      <c r="R10" s="6"/>
-      <c r="S10" s="6"/>
-      <c r="T10" s="6"/>
-      <c r="U10" s="6"/>
-      <c r="V10" s="6"/>
-      <c r="W10" s="6"/>
-      <c r="X10" s="6"/>
-      <c r="Y10" s="6"/>
-      <c r="Z10" s="6"/>
-      <c r="AA10" s="6"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="7"/>
-      <c r="B11" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C11" s="3" t="s">
+      <c r="H11" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="D11" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="E11" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="F11" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="G11" s="8">
-        <f t="shared" si="1"/>
-        <v>27</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>26</v>
       </c>
       <c r="I11" s="5">
         <v>46304.0</v>
@@ -1041,23 +1074,23 @@
         <v>3.0</v>
       </c>
       <c r="E12" s="4">
-        <v>5.0</v>
+        <v>3.0</v>
       </c>
       <c r="F12" s="4">
-        <v>5.0</v>
+        <v>3.0</v>
       </c>
       <c r="G12" s="8">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="I12" s="5">
         <v>46304.0</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K12" s="7"/>
       <c r="L12" s="3" t="s">
@@ -1080,36 +1113,34 @@
       <c r="AA12" s="6"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="7"/>
+      <c r="B13" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>59</v>
-      </c>
       <c r="D13" s="4">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="E13" s="4">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="F13" s="4">
         <v>5.0</v>
       </c>
       <c r="G13" s="8">
         <f t="shared" si="1"/>
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="I13" s="5">
         <v>46304.0</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K13" s="7"/>
       <c r="L13" s="3" t="s">
@@ -1132,7 +1163,9 @@
       <c r="AA13" s="6"/>
     </row>
     <row r="14">
-      <c r="A14" s="7"/>
+      <c r="A14" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="B14" s="2" t="s">
         <v>61</v>
       </c>
@@ -1146,11 +1179,11 @@
         <v>4.0</v>
       </c>
       <c r="F14" s="4">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="G14" s="8">
         <f t="shared" si="1"/>
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>26</v>
@@ -1183,24 +1216,24 @@
     </row>
     <row r="15">
       <c r="A15" s="7"/>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="2" t="s">
         <v>64</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>65</v>
       </c>
       <c r="D15" s="4">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="E15" s="4">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="F15" s="4">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="G15" s="8">
         <f t="shared" si="1"/>
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>26</v>
@@ -1232,36 +1265,34 @@
       <c r="AA15" s="6"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="7"/>
+      <c r="B16" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>69</v>
-      </c>
       <c r="D16" s="4">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="E16" s="4">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="F16" s="4">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="G16" s="8">
         <f t="shared" si="1"/>
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="I16" s="5">
         <v>46304.0</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K16" s="7"/>
       <c r="L16" s="3" t="s">
@@ -1284,7 +1315,9 @@
       <c r="AA16" s="6"/>
     </row>
     <row r="17">
-      <c r="A17" s="7"/>
+      <c r="A17" s="3" t="s">
+        <v>70</v>
+      </c>
       <c r="B17" s="2" t="s">
         <v>71</v>
       </c>
@@ -1484,36 +1517,34 @@
       <c r="AA20" s="6"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="7"/>
+      <c r="B21" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>85</v>
-      </c>
       <c r="D21" s="4">
         <v>3.0</v>
       </c>
       <c r="E21" s="4">
-        <v>5.0</v>
+        <v>2.0</v>
       </c>
       <c r="F21" s="4">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="G21" s="8">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>86</v>
+        <v>22</v>
       </c>
       <c r="I21" s="5">
         <v>46304.0</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="K21" s="7"/>
       <c r="L21" s="3" t="s">
@@ -1536,28 +1567,30 @@
       <c r="AA21" s="6"/>
     </row>
     <row r="22">
-      <c r="A22" s="3"/>
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
       <c r="B22" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>89</v>
-      </c>
       <c r="D22" s="4">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="E22" s="4">
-        <v>3.0</v>
+        <v>5.0</v>
       </c>
       <c r="F22" s="4">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
       <c r="G22" s="8">
         <f t="shared" si="1"/>
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="I22" s="5">
         <v>46304.0</v>
@@ -1594,20 +1627,20 @@
         <v>92</v>
       </c>
       <c r="D23" s="4">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="E23" s="4">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="F23" s="4">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="G23" s="8">
         <f t="shared" si="1"/>
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>22</v>
+        <v>89</v>
       </c>
       <c r="I23" s="5">
         <v>46304.0</v>
@@ -1636,36 +1669,34 @@
       <c r="AA23" s="6"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="3"/>
+      <c r="B24" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="C24" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>96</v>
-      </c>
       <c r="D24" s="4">
         <v>3.0</v>
       </c>
       <c r="E24" s="4">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="F24" s="4">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
       <c r="G24" s="8">
         <f t="shared" si="1"/>
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>97</v>
+        <v>22</v>
       </c>
       <c r="I24" s="5">
         <v>46304.0</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="K24" s="7"/>
       <c r="L24" s="3" t="s">
@@ -1689,16 +1720,16 @@
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C25" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B25" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>101</v>
-      </c>
       <c r="D25" s="4">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="E25" s="4">
         <v>3.0</v>
@@ -1708,16 +1739,16 @@
       </c>
       <c r="G25" s="8">
         <f t="shared" si="1"/>
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I25" s="5">
         <v>46304.0</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="K25" s="7"/>
       <c r="L25" s="3" t="s">
@@ -1740,18 +1771,41 @@
       <c r="AA25" s="6"/>
     </row>
     <row r="26">
-      <c r="A26" s="2"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="13"/>
-      <c r="J26" s="7"/>
+      <c r="A26" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="D26" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="E26" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="F26" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="G26" s="8">
+        <f t="shared" si="1"/>
+        <v>36</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="I26" s="5">
+        <v>46304.0</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>106</v>
+      </c>
       <c r="K26" s="7"/>
-      <c r="L26" s="7"/>
+      <c r="L26" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="M26" s="6"/>
       <c r="N26" s="6"/>
       <c r="O26" s="6"/>
@@ -1769,17 +1823,18 @@
       <c r="AA26" s="6"/>
     </row>
     <row r="27">
-      <c r="A27" s="14"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="15"/>
-      <c r="E27" s="16"/>
-      <c r="F27" s="16"/>
-      <c r="G27" s="16"/>
-      <c r="H27" s="6"/>
-      <c r="I27" s="17"/>
-      <c r="J27" s="18"/>
-      <c r="K27" s="6"/>
-      <c r="L27" s="6"/>
+      <c r="A27" s="2"/>
+      <c r="B27" s="10"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="20"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="7"/>
+      <c r="L27" s="7"/>
       <c r="M27" s="6"/>
       <c r="N27" s="6"/>
       <c r="O27" s="6"/>
@@ -1797,15 +1852,15 @@
       <c r="AA27" s="6"/>
     </row>
     <row r="28">
-      <c r="A28" s="14"/>
+      <c r="A28" s="21"/>
       <c r="C28" s="6"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="16"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="23"/>
       <c r="H28" s="6"/>
-      <c r="I28" s="17"/>
-      <c r="J28" s="6"/>
+      <c r="I28" s="24"/>
+      <c r="J28" s="25"/>
       <c r="K28" s="6"/>
       <c r="L28" s="6"/>
       <c r="M28" s="6"/>
@@ -1825,15 +1880,15 @@
       <c r="AA28" s="6"/>
     </row>
     <row r="29">
-      <c r="A29" s="6"/>
+      <c r="A29" s="21"/>
       <c r="C29" s="6"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23"/>
       <c r="H29" s="6"/>
-      <c r="I29" s="17"/>
-      <c r="J29" s="18"/>
+      <c r="I29" s="24"/>
+      <c r="J29" s="6"/>
       <c r="K29" s="6"/>
       <c r="L29" s="6"/>
       <c r="M29" s="6"/>
@@ -1855,15 +1910,15 @@
     <row r="30">
       <c r="A30" s="6"/>
       <c r="C30" s="6"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="16"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="23"/>
+      <c r="G30" s="23"/>
       <c r="H30" s="6"/>
-      <c r="I30" s="17"/>
-      <c r="J30" s="18"/>
-      <c r="K30" s="19"/>
-      <c r="L30" s="19"/>
+      <c r="I30" s="24"/>
+      <c r="J30" s="25"/>
+      <c r="K30" s="6"/>
+      <c r="L30" s="6"/>
       <c r="M30" s="6"/>
       <c r="N30" s="6"/>
       <c r="O30" s="6"/>
@@ -1883,13 +1938,13 @@
     <row r="31">
       <c r="A31" s="6"/>
       <c r="C31" s="6"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="16"/>
-      <c r="G31" s="16"/>
+      <c r="D31" s="23"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="23"/>
       <c r="H31" s="6"/>
-      <c r="I31" s="17"/>
-      <c r="J31" s="18"/>
+      <c r="I31" s="24"/>
+      <c r="J31" s="25"/>
       <c r="K31" s="6"/>
       <c r="L31" s="6"/>
       <c r="M31" s="6"/>
@@ -1911,15 +1966,15 @@
     <row r="32">
       <c r="A32" s="6"/>
       <c r="C32" s="6"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="16"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23"/>
+      <c r="G32" s="23"/>
       <c r="H32" s="6"/>
-      <c r="I32" s="17"/>
-      <c r="J32" s="18"/>
-      <c r="K32" s="19"/>
-      <c r="L32" s="19"/>
+      <c r="I32" s="24"/>
+      <c r="J32" s="25"/>
+      <c r="K32" s="6"/>
+      <c r="L32" s="6"/>
       <c r="M32" s="6"/>
       <c r="N32" s="6"/>
       <c r="O32" s="6"/>
@@ -1939,16 +1994,16 @@
     <row r="33">
       <c r="A33" s="6"/>
       <c r="C33" s="6"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="16"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="23"/>
       <c r="H33" s="6"/>
-      <c r="I33" s="17"/>
-      <c r="J33" s="18"/>
-      <c r="K33" s="19"/>
-      <c r="L33" s="19"/>
-      <c r="M33" s="19"/>
+      <c r="I33" s="24"/>
+      <c r="J33" s="25"/>
+      <c r="K33" s="6"/>
+      <c r="L33" s="6"/>
+      <c r="M33" s="6"/>
       <c r="N33" s="6"/>
       <c r="O33" s="6"/>
       <c r="P33" s="6"/>
@@ -1966,15 +2021,14 @@
     </row>
     <row r="34">
       <c r="A34" s="6"/>
-      <c r="B34" s="6"/>
       <c r="C34" s="6"/>
-      <c r="D34" s="6"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23"/>
+      <c r="G34" s="23"/>
       <c r="H34" s="6"/>
-      <c r="I34" s="6"/>
-      <c r="J34" s="6"/>
+      <c r="I34" s="24"/>
+      <c r="J34" s="25"/>
       <c r="K34" s="6"/>
       <c r="L34" s="6"/>
       <c r="M34" s="6"/>
@@ -1994,16 +2048,16 @@
       <c r="AA34" s="6"/>
     </row>
     <row r="35">
-      <c r="A35" s="7"/>
-      <c r="B35" s="7"/>
-      <c r="C35" s="7"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="16"/>
+      <c r="A35" s="6"/>
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
       <c r="G35" s="6"/>
       <c r="H35" s="6"/>
       <c r="I35" s="6"/>
-      <c r="J35" s="7"/>
+      <c r="J35" s="6"/>
       <c r="K35" s="6"/>
       <c r="L35" s="6"/>
       <c r="M35" s="6"/>
@@ -2026,9 +2080,9 @@
       <c r="A36" s="7"/>
       <c r="B36" s="7"/>
       <c r="C36" s="7"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="16"/>
-      <c r="F36" s="16"/>
+      <c r="D36" s="23"/>
+      <c r="E36" s="23"/>
+      <c r="F36" s="23"/>
       <c r="G36" s="6"/>
       <c r="H36" s="6"/>
       <c r="I36" s="6"/>
@@ -2055,9 +2109,9 @@
       <c r="A37" s="7"/>
       <c r="B37" s="7"/>
       <c r="C37" s="7"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16"/>
-      <c r="F37" s="16"/>
+      <c r="D37" s="23"/>
+      <c r="E37" s="23"/>
+      <c r="F37" s="23"/>
       <c r="G37" s="6"/>
       <c r="H37" s="6"/>
       <c r="I37" s="6"/>
@@ -2084,9 +2138,9 @@
       <c r="A38" s="7"/>
       <c r="B38" s="7"/>
       <c r="C38" s="7"/>
-      <c r="D38" s="16"/>
-      <c r="E38" s="16"/>
-      <c r="F38" s="16"/>
+      <c r="D38" s="23"/>
+      <c r="E38" s="23"/>
+      <c r="F38" s="23"/>
       <c r="G38" s="6"/>
       <c r="H38" s="6"/>
       <c r="I38" s="6"/>
@@ -2111,15 +2165,15 @@
     </row>
     <row r="39">
       <c r="A39" s="7"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="16"/>
-      <c r="F39" s="16"/>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="23"/>
+      <c r="E39" s="23"/>
+      <c r="F39" s="23"/>
       <c r="G39" s="6"/>
       <c r="H39" s="6"/>
       <c r="I39" s="6"/>
-      <c r="J39" s="7" t="s">
-        <v>104</v>
-      </c>
+      <c r="J39" s="7"/>
       <c r="K39" s="6"/>
       <c r="L39" s="6"/>
       <c r="M39" s="6"/>
@@ -2142,15 +2196,13 @@
       <c r="A40" s="7"/>
       <c r="B40" s="7"/>
       <c r="C40" s="7"/>
-      <c r="D40" s="16"/>
-      <c r="E40" s="16"/>
-      <c r="F40" s="16"/>
+      <c r="D40" s="23"/>
+      <c r="E40" s="6"/>
+      <c r="F40" s="6"/>
       <c r="G40" s="6"/>
       <c r="H40" s="6"/>
       <c r="I40" s="6"/>
-      <c r="J40" s="7" t="s">
-        <v>105</v>
-      </c>
+      <c r="J40" s="7"/>
       <c r="K40" s="6"/>
       <c r="L40" s="6"/>
       <c r="M40" s="6"/>
@@ -2170,16 +2222,16 @@
       <c r="AA40" s="6"/>
     </row>
     <row r="41">
-      <c r="A41" s="7"/>
-      <c r="B41" s="7"/>
-      <c r="C41" s="7"/>
-      <c r="D41" s="16"/>
+      <c r="A41" s="6"/>
+      <c r="B41" s="6"/>
+      <c r="C41" s="6"/>
+      <c r="D41" s="6"/>
       <c r="E41" s="6"/>
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
       <c r="H41" s="6"/>
       <c r="I41" s="6"/>
-      <c r="J41" s="7"/>
+      <c r="J41" s="6"/>
       <c r="K41" s="6"/>
       <c r="L41" s="6"/>
       <c r="M41" s="6"/>
@@ -2198,49 +2250,49 @@
       <c r="Z41" s="6"/>
       <c r="AA41" s="6"/>
     </row>
-    <row r="42">
-      <c r="A42" s="6"/>
-      <c r="B42" s="6"/>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
-      <c r="E42" s="6"/>
-      <c r="F42" s="6"/>
-      <c r="G42" s="6"/>
-      <c r="H42" s="6"/>
-      <c r="I42" s="6"/>
-      <c r="J42" s="6"/>
-      <c r="K42" s="6"/>
-      <c r="L42" s="6"/>
-      <c r="M42" s="6"/>
-      <c r="N42" s="6"/>
-      <c r="O42" s="6"/>
-      <c r="P42" s="6"/>
-      <c r="Q42" s="6"/>
-      <c r="R42" s="6"/>
-      <c r="S42" s="6"/>
-      <c r="T42" s="6"/>
-      <c r="U42" s="6"/>
-      <c r="V42" s="6"/>
-      <c r="W42" s="6"/>
-      <c r="X42" s="6"/>
-      <c r="Y42" s="6"/>
-      <c r="Z42" s="6"/>
-      <c r="AA42" s="6"/>
+    <row r="43">
+      <c r="A43" s="6"/>
+      <c r="B43" s="6"/>
+      <c r="C43" s="7"/>
+      <c r="D43" s="23"/>
+      <c r="E43" s="23"/>
+      <c r="F43" s="6"/>
+      <c r="G43" s="23"/>
+      <c r="H43" s="6"/>
+      <c r="I43" s="6"/>
+      <c r="J43" s="25"/>
+      <c r="K43" s="6"/>
+      <c r="L43" s="6"/>
+      <c r="M43" s="6"/>
+      <c r="N43" s="6"/>
+      <c r="O43" s="6"/>
+      <c r="P43" s="6"/>
+      <c r="Q43" s="6"/>
+      <c r="R43" s="6"/>
+      <c r="S43" s="6"/>
+      <c r="T43" s="6"/>
+      <c r="U43" s="6"/>
+      <c r="V43" s="6"/>
+      <c r="W43" s="6"/>
+      <c r="X43" s="6"/>
+      <c r="Y43" s="6"/>
+      <c r="Z43" s="6"/>
+      <c r="AA43" s="6"/>
     </row>
     <row r="44">
       <c r="A44" s="6"/>
       <c r="B44" s="6"/>
       <c r="C44" s="7"/>
-      <c r="D44" s="16"/>
-      <c r="E44" s="16"/>
+      <c r="D44" s="23"/>
+      <c r="E44" s="23"/>
       <c r="F44" s="6"/>
-      <c r="G44" s="16"/>
+      <c r="G44" s="23"/>
       <c r="H44" s="6"/>
       <c r="I44" s="6"/>
-      <c r="J44" s="18"/>
-      <c r="K44" s="19"/>
-      <c r="L44" s="19"/>
-      <c r="M44" s="19"/>
+      <c r="J44" s="25"/>
+      <c r="K44" s="6"/>
+      <c r="L44" s="6"/>
+      <c r="M44" s="6"/>
       <c r="N44" s="6"/>
       <c r="O44" s="6"/>
       <c r="P44" s="6"/>
@@ -2260,14 +2312,14 @@
       <c r="A45" s="6"/>
       <c r="B45" s="6"/>
       <c r="C45" s="7"/>
-      <c r="D45" s="16"/>
-      <c r="E45" s="16"/>
+      <c r="D45" s="23"/>
+      <c r="E45" s="23"/>
       <c r="F45" s="6"/>
-      <c r="G45" s="16"/>
+      <c r="G45" s="23"/>
       <c r="H45" s="6"/>
       <c r="I45" s="6"/>
-      <c r="J45" s="18"/>
-      <c r="K45" s="19"/>
+      <c r="J45" s="6"/>
+      <c r="K45" s="6"/>
       <c r="L45" s="6"/>
       <c r="M45" s="6"/>
       <c r="N45" s="6"/>
@@ -2289,10 +2341,10 @@
       <c r="A46" s="6"/>
       <c r="B46" s="6"/>
       <c r="C46" s="7"/>
-      <c r="D46" s="16"/>
-      <c r="E46" s="16"/>
+      <c r="D46" s="23"/>
+      <c r="E46" s="23"/>
       <c r="F46" s="6"/>
-      <c r="G46" s="16"/>
+      <c r="G46" s="23"/>
       <c r="H46" s="6"/>
       <c r="I46" s="6"/>
       <c r="J46" s="6"/>
@@ -2314,35 +2366,6 @@
       <c r="Z46" s="6"/>
       <c r="AA46" s="6"/>
     </row>
-    <row r="47">
-      <c r="A47" s="6"/>
-      <c r="B47" s="6"/>
-      <c r="C47" s="7"/>
-      <c r="D47" s="16"/>
-      <c r="E47" s="16"/>
-      <c r="F47" s="6"/>
-      <c r="G47" s="16"/>
-      <c r="H47" s="6"/>
-      <c r="I47" s="6"/>
-      <c r="J47" s="6"/>
-      <c r="K47" s="6"/>
-      <c r="L47" s="6"/>
-      <c r="M47" s="6"/>
-      <c r="N47" s="6"/>
-      <c r="O47" s="6"/>
-      <c r="P47" s="6"/>
-      <c r="Q47" s="6"/>
-      <c r="R47" s="6"/>
-      <c r="S47" s="6"/>
-      <c r="T47" s="6"/>
-      <c r="U47" s="6"/>
-      <c r="V47" s="6"/>
-      <c r="W47" s="6"/>
-      <c r="X47" s="6"/>
-      <c r="Y47" s="6"/>
-      <c r="Z47" s="6"/>
-      <c r="AA47" s="6"/>
-    </row>
   </sheetData>
   <drawing r:id="rId4"/>
   <legacyDrawing r:id="rId5"/>

</xml_diff>